<commit_message>
Dapine v3.0 FINAL - 84-step ultimate test, progress bars, timing, ML, 4 charts, bulletproof
</commit_message>
<xml_diff>
--- a/core_output.xlsx
+++ b/core_output.xlsx
@@ -59,9 +59,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>